<commit_message>
feat: sincroniza el catalogo de 93 fuentes
</commit_message>
<xml_diff>
--- a/centro-local/modules/medios/data/Medios_Matriz_Geopolitica_Navegacion_corregido.xlsx
+++ b/centro-local/modules/medios/data/Medios_Matriz_Geopolitica_Navegacion_corregido.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R239bcf31fdd848fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz profesional" sheetId="2" r:id="Rdec6f14def5c436f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodología" sheetId="3" r:id="R641db0388d94491a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Original" sheetId="4" r:id="Rab8f0368850a41bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura África" sheetId="5" r:id="R79f4902cde6d41bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Región" sheetId="6" r:id="Rd3d4377e4c7149ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Función" sheetId="7" r:id="R73fb0f1a00754aa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Perspectiva" sheetId="8" r:id="Re09cf0be6e774ce0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulta rápida" sheetId="9" r:id="R12adccb3dba746d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R26d67655b1e4471d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz profesional" sheetId="2" r:id="R64cedb75a79b4c4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodología" sheetId="3" r:id="R8fc906fb48264811"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Original" sheetId="4" r:id="Rf0fb99a224314174"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura África" sheetId="5" r:id="R0f64968c9d2c4b79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Región" sheetId="6" r:id="R558c358d66604682"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Función" sheetId="7" r:id="R9e31d173e23c4d52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Perspectiva" sheetId="8" r:id="Rc67c8fdff8ad46a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulta rápida" sheetId="9" r:id="Rbf458d6e36204b34"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1679,17 +1679,14 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr/>
               <a:t>Distribución por nivel de confianza</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
@@ -1807,17 +1804,14 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr/>
               <a:t>Distribución por estado de uso</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
@@ -1935,17 +1929,14 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr/>
               <a:t>Fuentes seleccionadas por subregión</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
@@ -2077,7 +2068,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rded7c19ead844c41"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb7c517d4863749ed"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2107,7 +2098,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R99c69f8947604740"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R09e201f83a8c4968"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2142,7 +2133,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R037fef8e3536497c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3caf40cd0702496d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2152,7 +2143,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MatrizFuentes" displayName="MatrizFuentes" ref="A4:AA96" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MatrizFuentes" displayName="MatrizFuentes" ref="A4:AA97" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="27">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Nombre"/>
@@ -2201,7 +2192,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TablaPorRegion" displayName="TablaPorRegion" ref="A4:AA96" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TablaPorRegion" displayName="TablaPorRegion" ref="A4:AA97" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="27">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Nombre"/>
@@ -2236,7 +2227,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TablaPorFuncion" displayName="TablaPorFuncion" ref="A4:AA96" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TablaPorFuncion" displayName="TablaPorFuncion" ref="A4:AA97" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="27">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Nombre"/>
@@ -2271,7 +2262,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TablaPorPerspectiva" displayName="TablaPorPerspectiva" ref="A4:AA96" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TablaPorPerspectiva" displayName="TablaPorPerspectiva" ref="A4:AA97" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="27">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Nombre"/>
@@ -2306,7 +2297,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TablaConsultaRapida" displayName="TablaConsultaRapida" ref="A4:L96" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TablaConsultaRapida" displayName="TablaConsultaRapida" ref="A4:L97" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Nombre"/>
     <x:tableColumn id="2" name="URL"/>
@@ -2368,9 +2359,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2539,8 +2530,7 @@
         <x:v>Total de fuentes</x:v>
       </x:c>
       <x:c r="B5" s="101" t="n">
-        <x:f>COUNTA('Matriz profesional'!B5:B96)</x:f>
-        <x:v>92</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D5" s="117" t="str">
         <x:v>Alta</x:v>
@@ -2569,15 +2559,13 @@
         <x:v>Media-alta</x:v>
       </x:c>
       <x:c r="E6" s="120" t="n">
-        <x:f>COUNTIF('Matriz profesional'!T5:T96,"Media-alta")</x:f>
-        <x:v>46</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="G6" s="129" t="str">
         <x:v>Nuevo recomendado</x:v>
       </x:c>
       <x:c r="H6" s="120" t="n">
-        <x:f>COUNTIF('Matriz profesional'!X5:X96,"Nuevo recomendado")</x:f>
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2854,7 +2842,7 @@
     <x:mergeCell ref="B34:J34"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e1ac28f01ab4a95"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8366f6259e294831"/>
 </x:worksheet>
 </file>
 
@@ -10748,6 +10736,89 @@
       </x:c>
       <x:c r="AA96" s="65" t="n">
         <x:v>46219</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>Geopolitical Futures</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>https://geopoliticalfutures.com/</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>Estados Unidos; sede en Austin, Texas; alcance global</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>Global/Occidente</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Inglés</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>Publicación especializada de análisis geopolítico</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>Análisis estratégico, prospectiva y evaluación de riesgos geopolíticos</x:v>
+      </x:c>
+      <x:c r="I97" t="str">
+        <x:v>Empresa privada; modelo de suscripción y apoyo de lectores</x:v>
+      </x:c>
+      <x:c r="J97" t="str">
+        <x:v>Privado</x:v>
+      </x:c>
+      <x:c r="K97" t="str">
+        <x:v>Realista / pragmático</x:v>
+      </x:c>
+      <x:c r="L97" t="str">
+        <x:v>Estadounidense / realista geoestratégica</x:v>
+      </x:c>
+      <x:c r="M97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O97" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="Q97" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="S97" t="n">
+        <x:v>3.7</x:v>
+      </x:c>
+      <x:c r="T97" t="str">
+        <x:v>Media-alta</x:v>
+      </x:c>
+      <x:c r="U97" t="str">
+        <x:v>Escenarios, análisis estructural y seguimiento de riesgos geopolíticos</x:v>
+      </x:c>
+      <x:c r="V97" t="str">
+        <x:v>Moderada-alta</x:v>
+      </x:c>
+      <x:c r="W97" t="str">
+        <x:v>Reuters/AP, fuentes primarias, think tanks de perspectivas distintas y medios locales</x:v>
+      </x:c>
+      <x:c r="X97" t="str">
+        <x:v>Nuevo recomendado</x:v>
+      </x:c>
+      <x:c r="Y97" t="str">
+        <x:v>Fundada por George Friedman. Ofrece análisis y previsiones mediante un modelo propio; sus interpretaciones y pronósticos deben contrastarse con datos, fuentes primarias y perspectivas regionales. No usar como confirmación única de hechos.</x:v>
+      </x:c>
+      <x:c r="Z97" t="str">
+        <x:v>https://geopoliticalfutures.com/analysis/</x:v>
+      </x:c>
+      <x:c r="AA97" t="n">
+        <x:v>46229</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10861,7 +10932,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R081cd06ec0ec4506"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5a001b784d544a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14174,9 +14245,9 @@
     <x:mergeCell ref="A38:H40"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd1fb80b30804b3b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18be216a45d64b75"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb1da85fbd154101"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd67d59710ec94782"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21889,6 +21960,89 @@
         <x:v>46219</x:v>
       </x:c>
     </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>Geopolitical Futures</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>https://geopoliticalfutures.com/</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>Estados Unidos; sede en Austin, Texas; alcance global</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>Global/Occidente</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Inglés</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>Publicación especializada de análisis geopolítico</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>Análisis estratégico, prospectiva y evaluación de riesgos geopolíticos</x:v>
+      </x:c>
+      <x:c r="I97" t="str">
+        <x:v>Empresa privada; modelo de suscripción y apoyo de lectores</x:v>
+      </x:c>
+      <x:c r="J97" t="str">
+        <x:v>Privado</x:v>
+      </x:c>
+      <x:c r="K97" t="str">
+        <x:v>Realista / pragmático</x:v>
+      </x:c>
+      <x:c r="L97" t="str">
+        <x:v>Estadounidense / realista geoestratégica</x:v>
+      </x:c>
+      <x:c r="M97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O97" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="Q97" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="S97" t="n">
+        <x:v>3.7</x:v>
+      </x:c>
+      <x:c r="T97" t="str">
+        <x:v>Media-alta</x:v>
+      </x:c>
+      <x:c r="U97" t="str">
+        <x:v>Escenarios, análisis estructural y seguimiento de riesgos geopolíticos</x:v>
+      </x:c>
+      <x:c r="V97" t="str">
+        <x:v>Moderada-alta</x:v>
+      </x:c>
+      <x:c r="W97" t="str">
+        <x:v>Reuters/AP, fuentes primarias, think tanks de perspectivas distintas y medios locales</x:v>
+      </x:c>
+      <x:c r="X97" t="str">
+        <x:v>Nuevo recomendado</x:v>
+      </x:c>
+      <x:c r="Y97" t="str">
+        <x:v>Fundada por George Friedman. Ofrece análisis y previsiones mediante un modelo propio; sus interpretaciones y pronósticos deben contrastarse con datos, fuentes primarias y perspectivas regionales. No usar como confirmación única de hechos.</x:v>
+      </x:c>
+      <x:c r="Z97" t="str">
+        <x:v>https://geopoliticalfutures.com/analysis/</x:v>
+      </x:c>
+      <x:c r="AA97" t="n">
+        <x:v>46229</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:AA1"/>
@@ -21896,7 +22050,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re52be2befda34517"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R854b35b2779e43ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29609,6 +29763,89 @@
         <x:v>46219</x:v>
       </x:c>
     </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>Geopolitical Futures</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>https://geopoliticalfutures.com/</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>Estados Unidos; sede en Austin, Texas; alcance global</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>Global/Occidente</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Inglés</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>Publicación especializada de análisis geopolítico</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>Análisis estratégico, prospectiva y evaluación de riesgos geopolíticos</x:v>
+      </x:c>
+      <x:c r="I97" t="str">
+        <x:v>Empresa privada; modelo de suscripción y apoyo de lectores</x:v>
+      </x:c>
+      <x:c r="J97" t="str">
+        <x:v>Privado</x:v>
+      </x:c>
+      <x:c r="K97" t="str">
+        <x:v>Realista / pragmático</x:v>
+      </x:c>
+      <x:c r="L97" t="str">
+        <x:v>Estadounidense / realista geoestratégica</x:v>
+      </x:c>
+      <x:c r="M97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O97" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="Q97" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="S97" t="n">
+        <x:v>3.7</x:v>
+      </x:c>
+      <x:c r="T97" t="str">
+        <x:v>Media-alta</x:v>
+      </x:c>
+      <x:c r="U97" t="str">
+        <x:v>Escenarios, análisis estructural y seguimiento de riesgos geopolíticos</x:v>
+      </x:c>
+      <x:c r="V97" t="str">
+        <x:v>Moderada-alta</x:v>
+      </x:c>
+      <x:c r="W97" t="str">
+        <x:v>Reuters/AP, fuentes primarias, think tanks de perspectivas distintas y medios locales</x:v>
+      </x:c>
+      <x:c r="X97" t="str">
+        <x:v>Nuevo recomendado</x:v>
+      </x:c>
+      <x:c r="Y97" t="str">
+        <x:v>Fundada por George Friedman. Ofrece análisis y previsiones mediante un modelo propio; sus interpretaciones y pronósticos deben contrastarse con datos, fuentes primarias y perspectivas regionales. No usar como confirmación única de hechos.</x:v>
+      </x:c>
+      <x:c r="Z97" t="str">
+        <x:v>https://geopoliticalfutures.com/analysis/</x:v>
+      </x:c>
+      <x:c r="AA97" t="n">
+        <x:v>46229</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:AA1"/>
@@ -29616,7 +29853,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc80fd973c1bb4c5b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd459cf22c2d04d20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37329,6 +37566,89 @@
         <x:v>46219</x:v>
       </x:c>
     </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>Geopolitical Futures</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>https://geopoliticalfutures.com/</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>Estados Unidos; sede en Austin, Texas; alcance global</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>Global/Occidente</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Inglés</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>Publicación especializada de análisis geopolítico</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>Análisis estratégico, prospectiva y evaluación de riesgos geopolíticos</x:v>
+      </x:c>
+      <x:c r="I97" t="str">
+        <x:v>Empresa privada; modelo de suscripción y apoyo de lectores</x:v>
+      </x:c>
+      <x:c r="J97" t="str">
+        <x:v>Privado</x:v>
+      </x:c>
+      <x:c r="K97" t="str">
+        <x:v>Realista / pragmático</x:v>
+      </x:c>
+      <x:c r="L97" t="str">
+        <x:v>Estadounidense / realista geoestratégica</x:v>
+      </x:c>
+      <x:c r="M97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O97" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="Q97" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R97" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="S97" t="n">
+        <x:v>3.7</x:v>
+      </x:c>
+      <x:c r="T97" t="str">
+        <x:v>Media-alta</x:v>
+      </x:c>
+      <x:c r="U97" t="str">
+        <x:v>Escenarios, análisis estructural y seguimiento de riesgos geopolíticos</x:v>
+      </x:c>
+      <x:c r="V97" t="str">
+        <x:v>Moderada-alta</x:v>
+      </x:c>
+      <x:c r="W97" t="str">
+        <x:v>Reuters/AP, fuentes primarias, think tanks de perspectivas distintas y medios locales</x:v>
+      </x:c>
+      <x:c r="X97" t="str">
+        <x:v>Nuevo recomendado</x:v>
+      </x:c>
+      <x:c r="Y97" t="str">
+        <x:v>Fundada por George Friedman. Ofrece análisis y previsiones mediante un modelo propio; sus interpretaciones y pronósticos deben contrastarse con datos, fuentes primarias y perspectivas regionales. No usar como confirmación única de hechos.</x:v>
+      </x:c>
+      <x:c r="Z97" t="str">
+        <x:v>https://geopoliticalfutures.com/analysis/</x:v>
+      </x:c>
+      <x:c r="AA97" t="n">
+        <x:v>46229</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:AA1"/>
@@ -37336,7 +37656,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R083edae0351e4b44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78d540c9d7974ee9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40925,6 +41245,44 @@
         <x:v>87</x:v>
       </x:c>
     </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>Geopolitical Futures</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>https://geopoliticalfutures.com/</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>Global/Occidente</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>Publicación especializada de análisis geopolítico</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>Análisis estratégico, prospectiva y evaluación de riesgos geopolíticos</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Estadounidense / realista geoestratégica</x:v>
+      </x:c>
+      <x:c r="G97" t="n">
+        <x:v>3.7</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>Media-alta</x:v>
+      </x:c>
+      <x:c r="I97" t="str">
+        <x:v>Escenarios, análisis estructural y seguimiento de riesgos geopolíticos</x:v>
+      </x:c>
+      <x:c r="J97" t="str">
+        <x:v>Moderada-alta</x:v>
+      </x:c>
+      <x:c r="K97" t="str">
+        <x:v>Nuevo recomendado</x:v>
+      </x:c>
+      <x:c r="L97" t="n">
+        <x:v>93</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:L1"/>
@@ -40932,7 +41290,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb01803bd74246db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d7ffa9101704361"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>